<commit_message>
chore: update  BRD and PRD file and add design
</commit_message>
<xml_diff>
--- a/docs/requirements/BRD_IEEE_29148_Checklist.xlsx
+++ b/docs/requirements/BRD_IEEE_29148_Checklist.xlsx
@@ -858,7 +858,7 @@
     <col customWidth="1" min="2" max="2" width="28"/>
     <col customWidth="1" min="3" max="3" width="68"/>
     <col customWidth="1" min="4" max="4" width="16"/>
-    <col customWidth="1" min="5" max="5" width="38"/>
+    <col customWidth="1" min="5" max="5" width="80"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -878,7 +878,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="28.5">
+    <row r="2" ht="81" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
@@ -888,12 +888,20 @@
       <c r="C2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="6"/>
-    </row>
-    <row r="3" ht="28.5">
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt] Vấn đề nghiệp vụ, nguyên nhân gốc và động lực được nêu tại mục 2 và 3.3–3.6 (nguồn SRC-001).
+Lưu ý: tác động chưa được định lượng (giờ/tuần, chi phí); lý do 'vì sao làm bây giờ' chưa rõ.
+Hành động: bổ sung số liệu khi có kết quả OQ-003, OQ-009.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="96" customHeight="1">
       <c r="A3" s="8"/>
       <c r="B3" s="9" t="s">
         <v>9</v>
@@ -901,12 +909,20 @@
       <c r="C3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="6"/>
-    </row>
-    <row r="4" ht="28.5">
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] Có 3 mục tiêu BO-001..003 và 3 KPI MET-001..003 kèm định nghĩa, công thức, nguồn dữ liệu, chủ sở hữu (mục 4).
+Thiếu: toàn bộ baseline/target đang [TBD]; chưa có kỳ vọng ROI / phân tích chi phí–lợi ích.
+Hành động: chốt OQ-003, OQ-005 (baseline, target), OQ-008 (ngân sách) và bổ sung ước tính ROI vào mục 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="66" customHeight="1">
       <c r="A4" s="8"/>
       <c r="B4" s="9" t="s">
         <v>11</v>
@@ -914,12 +930,19 @@
       <c r="C4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="6"/>
-    </row>
-    <row r="5" ht="28.5">
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt] Mục 5 nêu rõ trong phạm vi, ngoài phạm vi (kèm lý do), hạng mục hoãn và ranh giới.
+Lưu ý: các tính năng BA đề xuất (BR-016, BR-018, BR-021..023) còn chờ quản lý duyệt — OQ-013.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="81" customHeight="1">
       <c r="A5" s="10"/>
       <c r="B5" s="9" t="s">
         <v>13</v>
@@ -927,12 +950,19 @@
       <c r="C5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="6"/>
-    </row>
-    <row r="6" ht="28.5">
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Chưa đạt] BRD chưa có tuyên bố tầm nhìn (vision statement) riêng; mục 2 chỉ mô tả thay đổi đề xuất, chưa liên kết với chiến lược của tổ chức.
+Hành động: thêm 1–2 câu vision vào đầu mục 2, ví dụ: 'Mọi thành viên đội kinh doanh có được câu trả lời có nguồn kiểm chứng từ toàn bộ tài liệu dự án tại một nơi duy nhất'; xác nhận với sponsor sự liên kết chiến lược (thêm OQ mới).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="81" customHeight="1">
       <c r="A6" s="11" t="s">
         <v>15</v>
       </c>
@@ -942,12 +972,20 @@
       <c r="C6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="6"/>
-    </row>
-    <row r="7" ht="28.5">
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] Có 5 nhóm STK-001..005 với vai trò, mối quan tâm, mức ảnh hưởng (mục 6); đã nêu bên có thể chặn triển khai (STK-005).
+Thiếu: tên người cụ thể (OQ-001); bên liên quan bên ngoài như nhà cung cấp dịch vụ AI, chủ sở hữu/đối tác của tài liệu; STK-004, STK-005 mới là suy luận [Unverified].
+Hành động: bổ sung stakeholder bên ngoài và xác nhận danh sách với sponsor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="81" customHeight="1">
       <c r="A7" s="12"/>
       <c r="B7" s="9" t="s">
         <v>18</v>
@@ -955,12 +993,19 @@
       <c r="C7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="6"/>
-    </row>
-    <row r="8" ht="28.5">
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Chưa đạt] Mới chỉ có vai trò 'người dùng cuối' (STK-002); chưa mô tả hồ sơ người dùng: số lượng, mức độ thành thạo công nghệ/AI, bối cảnh làm việc, thiết bị, tần suất tra cứu, loại câu hỏi thường gặp.
+Hành động: phỏng vấn 3–5 người dùng đội kinh doanh (OQ-002, OQ-004) và thêm mục 'Hồ sơ người dùng' vào mục 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="96" customHeight="1">
       <c r="A8" s="13"/>
       <c r="B8" s="9" t="s">
         <v>20</v>
@@ -968,12 +1013,20 @@
       <c r="C8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="6"/>
-    </row>
-    <row r="9" ht="28.5">
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] CON-001..005 ghi nhận ràng buộc kỹ thuật (web, AI), tổ chức (MVP) và nghiệp vụ (PDF) — mục 9.
+Thiếu: ngân sách, thời hạn go-live (CON-005 đang [TBD]); chưa xác định ràng buộc pháp lý/quy định.
+Hành động: chốt OQ-008, OQ-009; bổ sung ràng buộc pháp lý sau khi review compliance (xem dòng 'Compliance &amp; Regulatory Standards').</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="51" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>22</v>
       </c>
@@ -983,12 +1036,19 @@
       <c r="C9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="6"/>
-    </row>
-    <row r="10" ht="28.5">
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt] Mục 3.1 có sơ đồ Mermaid quy trình hiện tại.
+Lưu ý: các bước được suy luận từ SRC-001 và đánh dấu [Unverified]; cần xác nhận qua phỏng vấn người dùng (OQ-002) trước khi baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="51" customHeight="1">
       <c r="A10" s="8"/>
       <c r="B10" s="9" t="s">
         <v>25</v>
@@ -996,12 +1056,19 @@
       <c r="C10" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="6"/>
-    </row>
-    <row r="11" ht="28.5">
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt] Mục 3.2 có sơ đồ quy trình đề xuất ở mức nghiệp vụ, thể hiện điểm cải tiến: hỏi một lần trên nhiều tài liệu, câu trả lời kèm nguồn để kiểm chứng.
+Gợi ý: thêm bảng so sánh As-Is/To-Be theo từng bước để thấy rõ bước nào được loại bỏ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="81" customHeight="1">
       <c r="A11" s="10"/>
       <c r="B11" s="9" t="s">
         <v>27</v>
@@ -1009,12 +1076,19 @@
       <c r="C11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="6"/>
-    </row>
-    <row r="12" ht="28.5">
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] Luồng To-Be và một số AC (vd. AC-015) gợi ý kịch bản sử dụng, nhưng BRD chưa có mục kịch bản vận hành / use case nghiệp vụ riêng.
+Hành động: bổ sung 3–5 kịch bản điển hình: (1) tra cứu thông tin nằm rải rác trong nhiều tài liệu; (2) hỏi thông tin không có trong tài liệu; (3) thay tài liệu cũ bằng phiên bản mới; (4) hỏi tiếp nhiều lượt để làm rõ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="96" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>29</v>
       </c>
@@ -1024,12 +1098,19 @@
       <c r="C12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" ht="28.5">
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] Các BR dùng cú pháp 'phải/nên/có thể' (shall/should/may), đã định nghĩa trong glossary; phần lớn mỗi BR chỉ một nghĩa vụ.
+Cần sửa: BR-002 gộp 2 điều kiện (sai định dạng; vượt dung lượng) → nên tách; BR-019 gộp 3 đối tượng (công cụ, tài liệu, câu trả lời) → tách hoặc định nghĩa thuật ngữ chung; BR-003 ('biết được khi nào') và BR-015 ('tham chiếu đến câu hỏi trước') cần diễn đạt cụ thể hơn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="81" customHeight="1">
       <c r="A13" s="12"/>
       <c r="B13" s="9" t="s">
         <v>32</v>
@@ -1037,12 +1118,20 @@
       <c r="C13" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="6"/>
-    </row>
-    <row r="14" ht="28.5">
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] Không có ngôn ngữ thiết kế/công nghệ trong BR; công nghệ chỉ xuất hiện ở ràng buộc (CON-001, CON-002) và ghi chú cho PRD (mục 15.2).
+Chưa đầy đủ: BR-001 (dung lượng), BR-012 (độ chính xác), BR-013 (thời gian phản hồi), BR-020 (chính sách dữ liệu) còn [TBD] — đều là Must.
+Hành động: chốt OQ-005, OQ-006, OQ-011, OQ-012.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="111" customHeight="1">
       <c r="A14" s="12"/>
       <c r="B14" s="9" t="s">
         <v>34</v>
@@ -1050,12 +1139,20 @@
       <c r="C14" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="6"/>
-    </row>
-    <row r="15" ht="28.5">
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] Mỗi BR có ID cố định, lý do, nguồn, AC; có ma trận truy vết và báo cáo độ phủ (mục 11).
+Không nhất quán: cột 'Nguồn' ở mục 7 của BR-002..006 và BR-014..020 chỉ ghi SN, nhưng ma trận mục 11 lại gán thêm BO → cần đồng bộ. Liên kết BR-019, BR-020 → BO-003 (mức độ sử dụng) còn yếu; nên thêm mục tiêu về bảo mật/tuân thủ hoặc chỉ truy vết về SN-009.
+SN-001, SN-008 không có BR riêng (đã ghi nhận trong báo cáo độ phủ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="96" customHeight="1">
       <c r="A15" s="13"/>
       <c r="B15" s="9" t="s">
         <v>36</v>
@@ -1063,12 +1160,20 @@
       <c r="C15" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="6"/>
-    </row>
-    <row r="16" ht="28.5">
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] Phạm vi MVP được giới hạn (CON-003, MoSCoW); rủi ro về khả thi đã nêu (RSK-004, RSK-005).
+Chưa có: đánh giá khả thi từ đội kỹ thuật; ngân sách/thời hạn chưa biết nên chưa kiểm được khả thi tổng thể. Một số AC có thể quá khắt khe với AI: AC-009 (0/10 câu chứa thông tin ngoài tài liệu), AC-011 (100% câu trả lời có trích dẫn).
+Hành động: đội kỹ thuật review khả thi; xác nhận ASM-001 bằng bộ tài liệu mẫu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="81" customHeight="1">
       <c r="A16" s="4" t="s">
         <v>38</v>
       </c>
@@ -1078,12 +1183,19 @@
       <c r="C16" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="6"/>
-    </row>
-    <row r="17" ht="28.5">
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Chưa đạt] Chỉ có BR-020 tham chiếu chung tới chính sách dữ liệu của tổ chức (đang [TBD: OQ-006]). Chưa xác định quy định pháp lý áp dụng (vd. quy định về bảo vệ dữ liệu cá nhân của Việt Nam nếu tài liệu chứa dữ liệu cá nhân), nghĩa vụ bảo mật theo hợp đồng với đối tác, và yêu cầu kiểm toán (ai tải lên / xóa / hỏi gì).
+Hành động: review với bộ phận pháp chế/bảo mật; bổ sung BR/CON và OQ tương ứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="66" customHeight="1">
       <c r="A17" s="8"/>
       <c r="B17" s="9" t="s">
         <v>41</v>
@@ -1091,12 +1203,19 @@
       <c r="C17" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" s="6"/>
-    </row>
-    <row r="18" ht="28.5">
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Chưa đạt] BRD chưa đề cập kỳ vọng về tính sẵn sàng (vd. trong giờ làm việc), thời gian gián đoạn chấp nhận được, RTO/RPO, và việc sao lưu/lưu giữ tài liệu đã tải lên.
+Hành động: thêm OQ cho sponsor về mức độ quan trọng của công cụ; ghi kết quả thành BR, hoặc ghi rõ 'không áp dụng cho MVP' kèm lý do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="96" customHeight="1">
       <c r="A18" s="10"/>
       <c r="B18" s="9" t="s">
         <v>43</v>
@@ -1104,12 +1223,20 @@
       <c r="C18" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" s="6"/>
-    </row>
-    <row r="19" ht="28.5">
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] Có BR-019 (chỉ người được cấp quyền truy cập), BR-020 (tuân thủ chính sách dữ liệu), BRU-005 (phạm vi chia sẻ tài liệu), RSK-002.
+Thiếu: chính sách lưu giữ/xóa dữ liệu (tài liệu, lịch sử hội thoại), ghi nhật ký truy cập, quyết định tài liệu riêng hay dùng chung (OQ-007), đánh giá việc gửi dữ liệu tới dịch vụ AI bên ngoài (OQ-006).
+Hành động: chốt OQ-006, OQ-007 và bổ sung quy tắc lưu giữ dữ liệu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="66" customHeight="1">
       <c r="A19" s="11" t="s">
         <v>45</v>
       </c>
@@ -1119,12 +1246,19 @@
       <c r="C19" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E19" s="6"/>
-    </row>
-    <row r="20" ht="28.5">
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt] ASM-001..004 được nêu rõ kèm tác động nếu sai, người chịu trách nhiệm, cách xác nhận và hạn (mục 10).
+Gợi ý bổ sung: giả định tài liệu tải lên là phiên bản mới nhất/chính xác; người dùng chấp nhận tự kiểm chứng câu trả lời qua nguồn trích dẫn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="66" customHeight="1">
       <c r="A20" s="12"/>
       <c r="B20" s="9" t="s">
         <v>48</v>
@@ -1132,12 +1266,19 @@
       <c r="C20" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E20" s="6"/>
-    </row>
-    <row r="21" ht="28.5">
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt] DEP-001..003 ghi nhận phụ thuộc vào dịch vụ AI, bộ tài liệu/câu hỏi chuẩn và hạ tầng (mục 10).
+Lưu ý: DEP-003 chưa có hạn (OQ-009); chưa nêu tường minh việc có/không có sáng kiến hay hệ thống liên quan — nên ghi rõ 'không có' nếu đúng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="96" customHeight="1">
       <c r="A21" s="13"/>
       <c r="B21" s="9" t="s">
         <v>50</v>
@@ -1145,10 +1286,18 @@
       <c r="C21" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E21" s="6"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Đạt một phần] RSK-001..006 được mô tả theo nguyên nhân → sự kiện → tác động, có mức độ nghiêm trọng, người chịu trách nhiệm và biện pháp giảm thiểu.
+Thiếu: kế hoạch dự phòng (contingency) khi rủi ro xảy ra, vd. RSK-001 vượt ngưỡng sai → hoãn go-live hoặc giới hạn phạm vi sử dụng; RSK-002 → quy trình xử lý sự cố lộ dữ liệu. Chưa đánh giá xác suất xảy ra.
+Hành động: bổ sung cột Xác suất và Kế hoạch dự phòng vào mục 10.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>